<commit_message>
Changed logic of interlock heartbeat sensing to account for cable capacitance
</commit_message>
<xml_diff>
--- a/doc/data packet structure.xlsx
+++ b/doc/data packet structure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rkiselev\Documents\dev\microsync\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E723593C-D3C0-460F-AA35-0B0B832B6477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1900DA49-D43D-4108-9533-7FB05497067E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8700" yWindow="1710" windowWidth="40620" windowHeight="17700" xr2:uid="{48FB7E95-C391-4754-94A5-34D8116DC883}"/>
+    <workbookView xWindow="22470" yWindow="2820" windowWidth="23865" windowHeight="17700" xr2:uid="{48FB7E95-C391-4754-94A5-34D8116DC883}"/>
   </bookViews>
   <sheets>
     <sheet name="Data packet format" sheetId="2" r:id="rId1"/>
@@ -1260,7 +1260,7 @@
     </r>
   </si>
   <si>
-    <t>v2.4.0</t>
+    <t>v2.6.x</t>
   </si>
 </sst>
 </file>
@@ -2891,6 +2891,15 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B32:K32"/>
+    <mergeCell ref="B33:K33"/>
+    <mergeCell ref="B34:K34"/>
+    <mergeCell ref="B35:K35"/>
+    <mergeCell ref="B27:K27"/>
+    <mergeCell ref="B28:K28"/>
+    <mergeCell ref="B29:K29"/>
+    <mergeCell ref="B30:K30"/>
+    <mergeCell ref="B31:K31"/>
     <mergeCell ref="B36:K36"/>
     <mergeCell ref="B44:K44"/>
     <mergeCell ref="B42:K42"/>
@@ -2900,19 +2909,19 @@
     <mergeCell ref="B37:K37"/>
     <mergeCell ref="B38:K38"/>
     <mergeCell ref="B39:K39"/>
-    <mergeCell ref="B32:K32"/>
-    <mergeCell ref="B33:K33"/>
-    <mergeCell ref="B34:K34"/>
-    <mergeCell ref="B35:K35"/>
-    <mergeCell ref="B27:K27"/>
-    <mergeCell ref="B28:K28"/>
-    <mergeCell ref="B29:K29"/>
-    <mergeCell ref="B30:K30"/>
-    <mergeCell ref="B31:K31"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="60" orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 St. Jude - Confidential</oddFooter>
+  </headerFooter>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{65ce1208-e929-4ec4-be64-9138d78922c0}" enabled="1" method="Standard" siteId="{22340fa8-9226-4871-b677-d3b3e377af72}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>